<commit_message>
Retire les tirets cadratins des figures et du classeur
Nettoyage etendu aux sorties visibles (les "---" de prose etaient deja traites) :
- 7 scripts de figures : tirets cadratins/demi-cadratins des titres, sous-titres,
  labels et prints remplaces par une ponctuation neutre (les separateurs de
  commentaires en traits d'union restent).
- figures F1, F3-F12 regenerees (F2 inchange : pas de tiret).
- cascade_piliers_DORA.xlsx regenere (titres de feuilles, marqueurs de cellules).
- fiche_pedagogique.pdf recompile (embarque F7, F11, F12).
Les figures Vasicek (G1/H1/J) : seul le texte source a change, sortie identique.
</commit_message>
<xml_diff>
--- a/exploratory/cascade_qualitative/cascade_piliers_DORA.xlsx
+++ b/exploratory/cascade_qualitative/cascade_piliers_DORA.xlsx
@@ -604,14 +604,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Combinaisons de piliers DORA — verdict qualitatif, l'ORDRE pilote</t>
+          <t>Combinaisons de piliers DORA : verdict qualitatif, l'ORDRE pilote</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Piliers : P1 = Gouvernance &amp; gestion du risque TIC  |  P2 = Gestion / classification / notification des incidents  |  P3 = Tests de résilience opérationnelle (TLPT)  |  P4 = Gestion du risque lié aux tiers ICT  |  P5 = Partage d'informations sur les cybermenaces   —   cascade cohérente (amont→aval) = probable ET grave ; à l'envers = rare et peu grave.</t>
+          <t>Piliers : P1 = Gouvernance &amp; gestion du risque TIC  |  P2 = Gestion / classification / notification des incidents  |  P3 = Tests de résilience opérationnelle (TLPT)  |  P4 = Gestion du risque lié aux tiers ICT  |  P5 = Partage d'informations sur les cybermenaces : cascade cohérente (amont→aval) = probable ET grave ; à l'envers = rare et peu grave.</t>
         </is>
       </c>
     </row>
@@ -692,22 +692,22 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I5" s="7" t="n"/>
@@ -28432,7 +28432,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Justification — comment l'ordre pilote le verdict (ancré DORA / mémoire)</t>
+          <t>Justification : comment l'ordre pilote le verdict (ancré DORA / mémoire)</t>
         </is>
       </c>
     </row>
@@ -28473,7 +28473,7 @@
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
         <is>
-          <t>GRAVITÉ (dépend de l'ordre — c'est le changement clé)</t>
+          <t>GRAVITÉ (dépend de l'ordre : c'est le changement clé)</t>
         </is>
       </c>
     </row>
@@ -28525,7 +28525,7 @@
     <row r="17">
       <c r="A17" s="29" t="inlineStr">
         <is>
-          <t>CRITICITÉ = moyenne géométrique( proba , gravité ) — croise likelihood et impact.</t>
+          <t>CRITICITÉ = moyenne géométrique( proba , gravité ) : croise likelihood et impact.</t>
         </is>
       </c>
     </row>
@@ -28535,7 +28535,7 @@
     <row r="19">
       <c r="A19" s="29" t="inlineStr">
         <is>
-          <t>Effet de l'ordre — exemple {P1,P2} :</t>
+          <t>Effet de l'ordre : exemple {P1,P2} :</t>
         </is>
       </c>
     </row>

</xml_diff>